<commit_message>
Stage 4: final memo, structured AI prompt, sensitivity expanded to ±10%
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/excel/Ferayorni-Alex-stage2-model-populated.xlsx
+++ b/docs/templates/excel/Ferayorni-Alex-stage2-model-populated.xlsx
@@ -439,7 +439,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -454,86 +454,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Main Model'!$C$51:$C$61</f>
-              <numCache>
-                <formatCode>0.0000</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$C$51:$C$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Main Model'!$D$51:$D$61</f>
-              <numCache>
-                <formatCode>\$#,##0;"($"#,##0\);\-</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$D$51:$D$71</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -587,7 +513,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -602,86 +528,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Main Model'!$C$51:$C$61</f>
-              <numCache>
-                <formatCode>0.0000</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$C$51:$C$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Main Model'!$E$51:$E$61</f>
-              <numCache>
-                <formatCode>\$#,##0;"($"#,##0\);\-</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$E$51:$E$71</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -735,7 +587,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -750,86 +602,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Main Model'!$C$51:$C$61</f>
-              <numCache>
-                <formatCode>0.0000</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$C$51:$C$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Main Model'!$F$51:$F$61</f>
-              <numCache>
-                <formatCode>\$#,##0;"($"#,##0\);\-</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$F$51:$F$71</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -883,7 +661,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -898,86 +676,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Main Model'!$C$51:$C$61</f>
-              <numCache>
-                <formatCode>0.0000</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$C$51:$C$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Main Model'!$G$51:$G$61</f>
-              <numCache>
-                <formatCode>\$#,##0;"($"#,##0\);\-</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$G$51:$G$71</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -1031,7 +735,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1046,86 +750,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Main Model'!$C$51:$C$61</f>
-              <numCache>
-                <formatCode>0.0000</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$C$51:$C$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Main Model'!$H$51:$H$61</f>
-              <numCache>
-                <formatCode>\$#,##0;"($"#,##0\);\-</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>0</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-                <pt idx="3">
-                  <v>0</v>
-                </pt>
-                <pt idx="4">
-                  <v>0</v>
-                </pt>
-                <pt idx="5">
-                  <v>0</v>
-                </pt>
-                <pt idx="6">
-                  <v>0</v>
-                </pt>
-                <pt idx="7">
-                  <v>0</v>
-                </pt>
-                <pt idx="8">
-                  <v>0</v>
-                </pt>
-                <pt idx="9">
-                  <v>0</v>
-                </pt>
-                <pt idx="10">
-                  <v>0</v>
-                </pt>
-              </numCache>
+              <f>'Main Model'!$H$51:$H$71</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -1218,7 +848,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1309,7 +939,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1342,7 +972,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1701,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2078,7 +1708,7 @@
     <row r="49" ht="21.75" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>5. SENSITIVITY  —  Ending spot rate S_T from 0.95×S0 to 1.05×S0</t>
+          <t>5. SENSITIVITY  —  Ending spot rate S_T from 0.90×S0 to 1.10×S0</t>
         </is>
       </c>
     </row>
@@ -2121,7 +1751,7 @@
     </row>
     <row r="51">
       <c r="B51" s="19" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="C51" s="13">
         <f>S0_in*(1+B51)</f>
@@ -2150,7 +1780,7 @@
     </row>
     <row r="52">
       <c r="B52" s="19" t="n">
-        <v>-0.04</v>
+        <v>-0.09</v>
       </c>
       <c r="C52" s="13">
         <f>S0_in*(1+B52)</f>
@@ -2179,7 +1809,7 @@
     </row>
     <row r="53">
       <c r="B53" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="C53" s="13">
         <f>S0_in*(1+B53)</f>
@@ -2208,7 +1838,7 @@
     </row>
     <row r="54">
       <c r="B54" s="19" t="n">
-        <v>-0.02</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="C54" s="13">
         <f>S0_in*(1+B54)</f>
@@ -2237,7 +1867,7 @@
     </row>
     <row r="55">
       <c r="B55" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.06</v>
       </c>
       <c r="C55" s="13">
         <f>S0_in*(1+B55)</f>
@@ -2266,7 +1896,7 @@
     </row>
     <row r="56">
       <c r="B56" s="19" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="C56" s="13">
         <f>S0_in*(1+B56)</f>
@@ -2295,7 +1925,7 @@
     </row>
     <row r="57">
       <c r="B57" s="19" t="n">
-        <v>0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="C57" s="13">
         <f>S0_in*(1+B57)</f>
@@ -2324,7 +1954,7 @@
     </row>
     <row r="58">
       <c r="B58" s="19" t="n">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="C58" s="13">
         <f>S0_in*(1+B58)</f>
@@ -2353,7 +1983,7 @@
     </row>
     <row r="59">
       <c r="B59" s="19" t="n">
-        <v>0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="C59" s="13">
         <f>S0_in*(1+B59)</f>
@@ -2382,7 +2012,7 @@
     </row>
     <row r="60">
       <c r="B60" s="19" t="n">
-        <v>0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="C60" s="13">
         <f>S0_in*(1+B60)</f>
@@ -2411,7 +2041,7 @@
     </row>
     <row r="61">
       <c r="B61" s="19" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="C61" s="13">
         <f>S0_in*(1+B61)</f>
@@ -2438,117 +2068,409 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="B62" s="19" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C62" s="13">
+        <f>S0_in*(1+B62)</f>
+        <v/>
+      </c>
+      <c r="D62" s="14">
+        <f>FC_AMT*C62</f>
+        <v/>
+      </c>
+      <c r="E62" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F62" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G62" s="14">
+        <f>MAX(K_PUT,C62)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H62" s="14">
+        <f>C62*FC_AMT+MAX(C62-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
     <row r="63" ht="31.5" customHeight="1">
-      <c r="B63" s="15" t="inlineStr">
+      <c r="B63" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C63" s="13">
+        <f>S0_in*(1+B63)</f>
+        <v/>
+      </c>
+      <c r="D63" s="14">
+        <f>FC_AMT*C63</f>
+        <v/>
+      </c>
+      <c r="E63" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F63" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G63" s="14">
+        <f>MAX(K_PUT,C63)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H63" s="14">
+        <f>C63*FC_AMT+MAX(C63-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C64" s="13">
+        <f>S0_in*(1+B64)</f>
+        <v/>
+      </c>
+      <c r="D64" s="14">
+        <f>FC_AMT*C64</f>
+        <v/>
+      </c>
+      <c r="E64" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F64" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G64" s="14">
+        <f>MAX(K_PUT,C64)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H64" s="14">
+        <f>C64*FC_AMT+MAX(C64-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="21.75" customHeight="1">
+      <c r="B65" s="19" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C65" s="13">
+        <f>S0_in*(1+B65)</f>
+        <v/>
+      </c>
+      <c r="D65" s="14">
+        <f>FC_AMT*C65</f>
+        <v/>
+      </c>
+      <c r="E65" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F65" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G65" s="14">
+        <f>MAX(K_PUT,C65)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H65" s="14">
+        <f>C65*FC_AMT+MAX(C65-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C66" s="13">
+        <f>S0_in*(1+B66)</f>
+        <v/>
+      </c>
+      <c r="D66" s="14">
+        <f>FC_AMT*C66</f>
+        <v/>
+      </c>
+      <c r="E66" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F66" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G66" s="14">
+        <f>MAX(K_PUT,C66)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H66" s="14">
+        <f>C66*FC_AMT+MAX(C66-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C67" s="13">
+        <f>S0_in*(1+B67)</f>
+        <v/>
+      </c>
+      <c r="D67" s="14">
+        <f>FC_AMT*C67</f>
+        <v/>
+      </c>
+      <c r="E67" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F67" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G67" s="14">
+        <f>MAX(K_PUT,C67)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H67" s="14">
+        <f>C67*FC_AMT+MAX(C67-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="19" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C68" s="13">
+        <f>S0_in*(1+B68)</f>
+        <v/>
+      </c>
+      <c r="D68" s="14">
+        <f>FC_AMT*C68</f>
+        <v/>
+      </c>
+      <c r="E68" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F68" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G68" s="14">
+        <f>MAX(K_PUT,C68)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H68" s="14">
+        <f>C68*FC_AMT+MAX(C68-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C69" s="13">
+        <f>S0_in*(1+B69)</f>
+        <v/>
+      </c>
+      <c r="D69" s="14">
+        <f>FC_AMT*C69</f>
+        <v/>
+      </c>
+      <c r="E69" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F69" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G69" s="14">
+        <f>MAX(K_PUT,C69)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H69" s="14">
+        <f>C69*FC_AMT+MAX(C69-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="19" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C70" s="13">
+        <f>S0_in*(1+B70)</f>
+        <v/>
+      </c>
+      <c r="D70" s="14">
+        <f>FC_AMT*C70</f>
+        <v/>
+      </c>
+      <c r="E70" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F70" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G70" s="14">
+        <f>MAX(K_PUT,C70)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H70" s="14">
+        <f>C70*FC_AMT+MAX(C70-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C71" s="13">
+        <f>S0_in*(1+B71)</f>
+        <v/>
+      </c>
+      <c r="D71" s="14">
+        <f>FC_AMT*C71</f>
+        <v/>
+      </c>
+      <c r="E71" s="14">
+        <f>FC_AMT*F0_in</f>
+        <v/>
+      </c>
+      <c r="F71" s="14">
+        <f>$C$34</f>
+        <v/>
+      </c>
+      <c r="G71" s="14">
+        <f>MAX(K_PUT,C71)*FC_AMT-$C$41</f>
+        <v/>
+      </c>
+      <c r="H71" s="14">
+        <f>C71*FC_AMT+MAX(C71-K_CALL,0)*FC_AMT-$C$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72"/>
+    <row r="73">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>Notes: Forward and Money Market columns are flat (locked-in). Put floors downside below K_PUT. Call column shows unhedged receivable PLUS long call — this is a speculative structure, not a hedge, shown here per request for side-by-side comparison with the put.</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="21.75" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="74"/>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>6. SUMMARY OUTPUTS  (KPIs)</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="7" t="inlineStr">
+    <row r="76">
+      <c r="B76" s="7" t="inlineStr">
         <is>
           <t>Forward hedge — USD proceeds</t>
         </is>
       </c>
-      <c r="C66" s="20">
+      <c r="C76" s="20">
         <f>C26</f>
         <v/>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" s="7" t="inlineStr">
+    <row r="77">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>Money Market hedge — USD proceeds</t>
         </is>
       </c>
-      <c r="C67" s="20">
+      <c r="C77" s="20">
         <f>C34</f>
         <v/>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" s="7" t="inlineStr">
+    <row r="78">
+      <c r="B78" s="7" t="inlineStr">
         <is>
           <t>Put on EUR — USD proceeds at S0 (at-the-money view)</t>
         </is>
       </c>
-      <c r="C68" s="20">
+      <c r="C78" s="20">
         <f>MAX(K_PUT,S0_in)*FC_AMT-C41</f>
         <v/>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="7" t="inlineStr">
+    <row r="79">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>Put on EUR — USD proceeds if S_T = K_PUT (floor)</t>
         </is>
       </c>
-      <c r="C69" s="20">
+      <c r="C79" s="20">
         <f>K_PUT*FC_AMT-C41</f>
         <v/>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" s="7" t="inlineStr">
+    <row r="80">
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>Call on EUR — USD proceeds at S0  (comparison, not a hedge)</t>
         </is>
       </c>
-      <c r="C70" s="20">
+      <c r="C80" s="20">
         <f>S0_in*FC_AMT+MAX(S0_in-K_CALL,0)*FC_AMT-C43</f>
         <v/>
       </c>
     </row>
-    <row r="71">
-      <c r="B71" s="7" t="inlineStr">
+    <row r="81">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>Unhedged — USD proceeds at current spot</t>
         </is>
       </c>
-      <c r="C71" s="20">
+      <c r="C81" s="20">
         <f>S0_in*FC_AMT</f>
         <v/>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" s="7" t="inlineStr">
+    <row r="82">
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>HEDGE RECOMMENDATION  (to be completed in Stage 4)</t>
         </is>
       </c>
-      <c r="C72" s="1" t="n"/>
-      <c r="D72" s="23" t="n"/>
-      <c r="E72" s="23" t="n"/>
-      <c r="F72" s="23" t="n"/>
-      <c r="G72" s="23" t="n"/>
-      <c r="H72" s="24" t="n"/>
+      <c r="C82" s="1" t="n"/>
+      <c r="D82" s="23" t="n"/>
+      <c r="E82" s="23" t="n"/>
+      <c r="F82" s="23" t="n"/>
+      <c r="G82" s="23" t="n"/>
+      <c r="H82" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="C82:H82"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A15:F15"/>
     <mergeCell ref="A49:F49"/>
-    <mergeCell ref="C72:H72"/>
     <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="B63:H63"/>
+    <mergeCell ref="B73:H73"/>
+    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>